<commit_message>
Update agro sector (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/agro sector (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/agro sector (VDS_s) 0.xlsx
@@ -12,7 +12,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="inf16" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
@@ -88,6 +88,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>

</xml_diff>